<commit_message>
Fixed some Design bugs
added some pdfs
</commit_message>
<xml_diff>
--- a/8Bit Computer ver2.0/excel/chips availability.xlsx
+++ b/8Bit Computer ver2.0/excel/chips availability.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\home\Desktop\Computer_HTL\8Bit Computer ver2.0\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967F6007-B5AD-420D-ABEC-138A5DFC9508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD18090-2B93-4BF9-B860-970F175465CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E9CC7EE1-7E8B-4FEA-8BE1-446B4A860683}"/>
+    <workbookView xWindow="-25320" yWindow="315" windowWidth="25440" windowHeight="15270" xr2:uid="{E9CC7EE1-7E8B-4FEA-8BE1-446B4A860683}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="249">
   <si>
     <t>Boolean Logic</t>
   </si>
@@ -202,9 +202,6 @@
   </si>
   <si>
     <t>use</t>
-  </si>
-  <si>
-    <t>need Invert for clk</t>
   </si>
   <si>
     <t>Info</t>
@@ -463,9 +460,6 @@
   </si>
   <si>
     <t>1.6EUR</t>
-  </si>
-  <si>
-    <t>use need Invert for clk</t>
   </si>
   <si>
     <t>2x</t>
@@ -526,9 +520,6 @@
       </rPr>
       <t>/HCS</t>
     </r>
-  </si>
-  <si>
-    <t>for clk</t>
   </si>
   <si>
     <t>74x1G08</t>
@@ -1602,10 +1593,10 @@
     </row>
     <row r="2" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>1</v>
@@ -1614,19 +1605,19 @@
         <v>9</v>
       </c>
       <c r="F2" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="G2" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="G2" s="12" t="s">
-        <v>88</v>
-      </c>
       <c r="H2" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="I2" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="I2" s="12" t="s">
-        <v>78</v>
-      </c>
       <c r="J2" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K2" s="11" t="s">
         <v>2</v>
@@ -1636,22 +1627,22 @@
       </c>
       <c r="M2" s="14"/>
       <c r="N2" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="O2" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="O2" s="12" t="s">
-        <v>80</v>
-      </c>
       <c r="P2" s="12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q2" s="12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>33</v>
@@ -1660,7 +1651,7 @@
         <v>3</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="3"/>
@@ -1675,41 +1666,41 @@
         <v>55</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H4" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H4" s="28" t="s">
+      <c r="I4" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="I4" s="17" t="s">
-        <v>78</v>
-      </c>
       <c r="J4" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K4" s="27" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L4" s="1"/>
       <c r="N4" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="O4" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="O4" s="17" t="s">
-        <v>80</v>
-      </c>
       <c r="P4" s="26" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q4" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="2:17" x14ac:dyDescent="0.25">
@@ -1718,41 +1709,41 @@
         <v>55</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H5" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I5" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="I5" s="20" t="s">
-        <v>78</v>
-      </c>
       <c r="J5" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K5" s="27" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L5" s="1"/>
       <c r="N5" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="O5" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="O5" s="20" t="s">
-        <v>80</v>
-      </c>
       <c r="P5" s="26" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q5" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="2:17" x14ac:dyDescent="0.25">
@@ -1767,35 +1758,35 @@
         <v>4</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H6" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="I6" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="I6" s="17" t="s">
-        <v>78</v>
-      </c>
       <c r="J6" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K6" s="27" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L6" s="1"/>
       <c r="N6" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="O6" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="O6" s="17" t="s">
-        <v>80</v>
-      </c>
       <c r="P6" s="26" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q6" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="2:17" x14ac:dyDescent="0.25">
@@ -1810,35 +1801,35 @@
         <v>5</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H7" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="I7" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="I7" s="17" t="s">
-        <v>78</v>
-      </c>
       <c r="J7" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K7" s="27" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L7" s="1"/>
       <c r="N7" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="O7" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="O7" s="17" t="s">
-        <v>80</v>
-      </c>
       <c r="P7" s="26" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q7" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="2:17" x14ac:dyDescent="0.25">
@@ -1853,35 +1844,35 @@
         <v>6</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H8" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="I8" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="I8" s="17" t="s">
-        <v>78</v>
-      </c>
       <c r="J8" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K8" s="27" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L8" s="1"/>
       <c r="N8" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="O8" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="O8" s="17" t="s">
-        <v>80</v>
-      </c>
       <c r="P8" s="26" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q8" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="2:17" x14ac:dyDescent="0.25">
@@ -1889,44 +1880,44 @@
         <v>6</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>5</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H9" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I9" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="I9" s="20" t="s">
-        <v>78</v>
-      </c>
       <c r="J9" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K9" s="27" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L9" s="1"/>
       <c r="N9" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="O9" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="O9" s="20" t="s">
-        <v>80</v>
-      </c>
       <c r="P9" s="26" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q9" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.25">
@@ -1934,44 +1925,44 @@
         <v>2</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>5</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H10" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I10" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="I10" s="20" t="s">
-        <v>78</v>
-      </c>
       <c r="J10" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K10" s="27" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L10" s="1"/>
       <c r="N10" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="O10" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="O10" s="20" t="s">
-        <v>80</v>
-      </c>
       <c r="P10" s="26" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q10" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.25">
@@ -1980,35 +1971,35 @@
         <v>55</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="1" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="K11" s="22" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="L11" s="1"/>
       <c r="N11" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O11" s="1"/>
       <c r="P11" s="26" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q11" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="2:17" x14ac:dyDescent="0.25">
@@ -2017,70 +2008,70 @@
         <v>55</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="1" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="K12" s="22" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="L12" s="1"/>
       <c r="N12" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O12" s="1"/>
       <c r="P12" s="26" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q12" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
       <c r="C13" s="15"/>
       <c r="D13" s="1" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="1" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="K13" s="22" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="L13" s="1"/>
       <c r="N13" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O13" s="1"/>
       <c r="P13" s="31" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="Q13" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="14" spans="2:17" x14ac:dyDescent="0.25">
@@ -2118,7 +2109,7 @@
     <row r="16" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
       <c r="C16" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>1</v>
@@ -2127,14 +2118,14 @@
         <v>9</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G16" s="13"/>
       <c r="H16" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="I16" s="12" t="s">
         <v>77</v>
-      </c>
-      <c r="I16" s="12" t="s">
-        <v>78</v>
       </c>
       <c r="J16" s="11" t="s">
         <v>8</v>
@@ -2146,13 +2137,13 @@
         <v>20</v>
       </c>
       <c r="N16" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="O16" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="O16" s="12" t="s">
-        <v>80</v>
-      </c>
       <c r="P16" s="12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q16" s="1"/>
     </row>
@@ -2165,10 +2156,10 @@
         <v>34</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G17" s="7"/>
       <c r="H17" s="10" t="s">
@@ -2196,10 +2187,10 @@
         <v>35</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G18" s="7"/>
       <c r="H18" s="10" t="s">
@@ -2227,10 +2218,10 @@
         <v>37</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G19" s="7"/>
       <c r="H19" s="10" t="s">
@@ -2258,53 +2249,53 @@
         <v>41</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H20" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="I20" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="I20" s="18" t="s">
-        <v>78</v>
-      </c>
       <c r="J20" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>29</v>
       </c>
       <c r="L20" s="1"/>
       <c r="N20" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="O20" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="O20" s="18" t="s">
-        <v>80</v>
-      </c>
       <c r="P20" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q20" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B21" s="1"/>
       <c r="C21" s="16" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="G21" s="1"/>
       <c r="H21" s="20" t="s">
@@ -2312,10 +2303,10 @@
       </c>
       <c r="I21" s="18"/>
       <c r="J21" s="1" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="L21" s="1"/>
       <c r="N21" s="20" t="s">
@@ -2323,10 +2314,10 @@
       </c>
       <c r="O21" s="18"/>
       <c r="P21" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q21" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="2:17" x14ac:dyDescent="0.25">
@@ -2334,36 +2325,36 @@
         <v>1</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G22" s="1"/>
       <c r="H22" s="20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I22" s="18"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L22" s="1"/>
       <c r="N22" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O22" s="18"/>
       <c r="P22" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q22" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="23" spans="2:17" x14ac:dyDescent="0.25">
@@ -2378,30 +2369,30 @@
         <v>21</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G23" s="1"/>
       <c r="H23" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I23" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="I23" s="17" t="s">
-        <v>78</v>
-      </c>
       <c r="J23" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="L23" s="1"/>
       <c r="N23" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="O23" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="O23" s="21" t="s">
-        <v>80</v>
-      </c>
       <c r="P23" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q23" s="1"/>
     </row>
@@ -2411,28 +2402,28 @@
         <v>50</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G24" s="1"/>
       <c r="H24" s="20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I24" s="17"/>
       <c r="J24" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K24" s="22" t="s">
         <v>29</v>
       </c>
       <c r="L24" s="1"/>
       <c r="N24" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O24" s="21"/>
       <c r="Q24" s="17"/>
@@ -2441,17 +2432,17 @@
       <c r="B25" s="1">
         <v>1</v>
       </c>
-      <c r="C25" s="16" t="s">
-        <v>146</v>
+      <c r="C25" s="23" t="s">
+        <v>50</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="F25" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G25" s="1"/>
       <c r="H25" s="20" t="s">
@@ -2460,7 +2451,7 @@
       <c r="I25" s="17"/>
       <c r="J25" s="1"/>
       <c r="K25" s="22" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L25" s="1"/>
       <c r="N25" s="20" t="s">
@@ -2468,10 +2459,10 @@
       </c>
       <c r="O25" s="21"/>
       <c r="P25" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q25" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="26" spans="2:17" x14ac:dyDescent="0.25">
@@ -2480,13 +2471,13 @@
         <v>50</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G26" s="7"/>
       <c r="H26" s="10" t="s">
@@ -2499,7 +2490,7 @@
       </c>
       <c r="L26" s="7"/>
       <c r="M26" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="N26" s="10" t="s">
         <v>51</v>
@@ -2520,7 +2511,7 @@
         <v>21</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G27" s="7"/>
       <c r="H27" s="10" t="s">
@@ -2548,10 +2539,10 @@
         <v>38</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G28" s="7"/>
       <c r="H28" s="7" t="s">
@@ -2573,42 +2564,42 @@
     <row r="29" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
       <c r="C29" s="16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>39</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G29" s="1"/>
       <c r="H29" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I29" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="I29" s="20" t="s">
-        <v>78</v>
-      </c>
       <c r="J29" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="L29" s="1"/>
       <c r="N29" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="O29" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="O29" s="20" t="s">
-        <v>80</v>
-      </c>
       <c r="P29" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q29" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" spans="2:17" x14ac:dyDescent="0.25">
@@ -2678,10 +2669,10 @@
         <v>46</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G32" s="7"/>
       <c r="H32" s="7"/>
@@ -2707,10 +2698,10 @@
         <v>48</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G33" s="7"/>
       <c r="H33" s="7"/>
@@ -2729,37 +2720,37 @@
     </row>
     <row r="34" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C34" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H34" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="J34" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="K34" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="L34" t="s">
         <v>151</v>
       </c>
-      <c r="F34" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="H34" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="K34" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="L34" t="s">
-        <v>154</v>
-      </c>
       <c r="N34" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P34" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q34" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="35" spans="2:18" x14ac:dyDescent="0.25">
@@ -2767,25 +2758,25 @@
         <v>55</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="H35" s="39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K35" s="22" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N35" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P35" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q35" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="36" spans="2:18" x14ac:dyDescent="0.25">
@@ -2856,7 +2847,7 @@
     <row r="41" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B41" s="1"/>
       <c r="C41" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D41" s="11" t="s">
         <v>1</v>
@@ -2877,10 +2868,10 @@
         <v>2</v>
       </c>
       <c r="L41" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M41" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N41" s="11" t="s">
         <v>51</v>
@@ -2893,13 +2884,13 @@
         <v>50</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G42" s="1"/>
       <c r="H42" s="5" t="s">
@@ -2909,7 +2900,7 @@
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
       <c r="L42" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="N42" s="5" t="s">
         <v>51</v>
@@ -2919,16 +2910,16 @@
     <row r="43" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B43" s="1"/>
       <c r="C43" s="19" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="G43" s="1"/>
       <c r="H43" s="5" t="s">
@@ -2936,20 +2927,20 @@
       </c>
       <c r="I43" s="5"/>
       <c r="J43" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K43" s="1"/>
       <c r="L43" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="N43" s="5" t="s">
         <v>51</v>
       </c>
       <c r="P43" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q43" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="44" spans="2:18" x14ac:dyDescent="0.25">
@@ -2958,13 +2949,13 @@
         <v>50</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E44" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="5" t="s">
@@ -2972,20 +2963,20 @@
       </c>
       <c r="I44" s="5"/>
       <c r="J44" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K44" s="1"/>
       <c r="L44" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="N44" s="5" t="s">
         <v>51</v>
       </c>
       <c r="P44" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q44" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="45" spans="2:18" x14ac:dyDescent="0.25">
@@ -2996,13 +2987,13 @@
         <v>50</v>
       </c>
       <c r="D45" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="G45" s="1"/>
       <c r="H45" s="5" t="s">
@@ -3010,23 +3001,23 @@
       </c>
       <c r="I45" s="1"/>
       <c r="J45" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K45" s="1"/>
       <c r="L45" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M45" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N45" s="5" t="s">
         <v>51</v>
       </c>
       <c r="P45" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q45" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="46" spans="2:18" x14ac:dyDescent="0.25">
@@ -3037,13 +3028,13 @@
         <v>55</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G46" s="1"/>
       <c r="H46" s="5" t="s">
@@ -3051,23 +3042,23 @@
       </c>
       <c r="I46" s="1"/>
       <c r="J46" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K46" s="1"/>
       <c r="L46" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M46" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N46" s="5" t="s">
         <v>51</v>
       </c>
       <c r="P46" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q46" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="47" spans="2:18" x14ac:dyDescent="0.25">
@@ -3078,13 +3069,13 @@
         <v>50</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E47" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F47" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>121</v>
       </c>
       <c r="G47" s="1"/>
       <c r="H47" s="5" t="s">
@@ -3092,7 +3083,7 @@
       </c>
       <c r="I47" s="1"/>
       <c r="J47" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
@@ -3100,7 +3091,7 @@
         <v>51</v>
       </c>
       <c r="Q47" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="48" spans="2:18" x14ac:dyDescent="0.25">
@@ -3111,46 +3102,46 @@
         <v>55</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H48" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I48" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="N48" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O48" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="P48" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q48" s="5" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="R48" s="5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="49" spans="2:18" x14ac:dyDescent="0.25">
@@ -3158,62 +3149,62 @@
         <v>55</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G49" s="1"/>
       <c r="H49" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I49" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="L49" s="1"/>
       <c r="N49" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O49" s="21" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="P49" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q49" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R49" s="5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="50" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B50" s="1">
         <v>9</v>
       </c>
-      <c r="C50" s="16" t="s">
-        <v>56</v>
+      <c r="C50" s="23" t="s">
+        <v>50</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H50" s="17" t="s">
         <v>7</v>
@@ -3227,48 +3218,48 @@
         <v>51</v>
       </c>
       <c r="P50" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q50" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="51" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
-      <c r="C51" s="19" t="s">
-        <v>131</v>
+      <c r="C51" s="23" t="s">
+        <v>50</v>
       </c>
       <c r="D51" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E51" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="G51" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H51" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I51" s="3"/>
       <c r="J51" s="24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="L51" s="1"/>
       <c r="N51" s="5" t="s">
         <v>51</v>
       </c>
       <c r="P51" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q51" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="52" spans="2:18" x14ac:dyDescent="0.25">
@@ -3279,13 +3270,13 @@
         <v>55</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="G52" s="1"/>
       <c r="H52" s="5" t="s">
@@ -3293,98 +3284,98 @@
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="24" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L52" s="24" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="N52" s="5" t="s">
         <v>51</v>
       </c>
       <c r="P52" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q52" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="53" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
       <c r="C53" s="19" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H53" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I53" s="3"/>
       <c r="J53" s="24" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="L53" s="24"/>
       <c r="N53" s="5" t="s">
         <v>51</v>
       </c>
       <c r="P53" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q53" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="54" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B54" s="1"/>
-      <c r="C54" s="19" t="s">
+      <c r="C54" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="D54" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="D54" s="1" t="s">
-        <v>179</v>
-      </c>
       <c r="E54" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H54" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I54" s="3"/>
       <c r="J54" s="24" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="L54" s="24"/>
       <c r="N54" s="5" t="s">
         <v>51</v>
       </c>
       <c r="P54" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q54" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="55" spans="2:18" ht="21" x14ac:dyDescent="0.35">
@@ -3403,7 +3394,7 @@
     </row>
     <row r="56" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C56" s="13" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>1</v>
@@ -3453,13 +3444,13 @@
     <row r="58" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C58" s="29"/>
       <c r="D58" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="E58" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="E58" s="15" t="s">
-        <v>190</v>
-      </c>
       <c r="F58" s="15" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="G58" s="15"/>
       <c r="H58" s="30"/>
@@ -3473,23 +3464,23 @@
       </c>
       <c r="O58" s="29"/>
       <c r="P58" s="31" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="Q58" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R58" s="29"/>
     </row>
     <row r="59" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C59" s="29"/>
       <c r="D59" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="E59" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="F59" s="15" t="s">
         <v>188</v>
-      </c>
-      <c r="E59" s="15" t="s">
-        <v>189</v>
-      </c>
-      <c r="F59" s="15" t="s">
-        <v>191</v>
       </c>
       <c r="G59" s="15"/>
       <c r="H59" s="30"/>
@@ -3503,23 +3494,23 @@
       </c>
       <c r="O59" s="29"/>
       <c r="P59" s="31" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="Q59" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R59" s="29"/>
     </row>
     <row r="60" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C60" s="29"/>
       <c r="D60" s="15" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="E60" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="F60" s="15" t="s">
         <v>190</v>
-      </c>
-      <c r="F60" s="15" t="s">
-        <v>193</v>
       </c>
       <c r="G60" s="15"/>
       <c r="H60" s="30"/>
@@ -3533,23 +3524,23 @@
       </c>
       <c r="O60" s="29"/>
       <c r="P60" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q60" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R60" s="29"/>
     </row>
     <row r="61" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C61" s="29"/>
       <c r="D61" s="15" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E61" s="15" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="F61" s="15" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="G61" s="15"/>
       <c r="H61" s="30"/>
@@ -3563,23 +3554,23 @@
       </c>
       <c r="O61" s="29"/>
       <c r="P61" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q61" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R61" s="29"/>
     </row>
     <row r="62" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C62" s="29"/>
       <c r="D62" s="15" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="E62" s="15" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F62" s="15" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="G62" s="15"/>
       <c r="H62" s="30"/>
@@ -3589,7 +3580,7 @@
         <v>-20</v>
       </c>
       <c r="L62" s="15" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="M62" s="29"/>
       <c r="N62" s="20" t="s">
@@ -3597,22 +3588,22 @@
       </c>
       <c r="O62" s="29"/>
       <c r="P62" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q62" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R62" s="29"/>
     </row>
     <row r="63" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C63" s="29" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D63" s="15" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E63" s="15" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="F63" s="15"/>
       <c r="G63" s="15"/>
@@ -3627,20 +3618,20 @@
       </c>
       <c r="O63" s="29"/>
       <c r="P63" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q63" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R63" s="29"/>
     </row>
     <row r="64" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C64" s="29"/>
       <c r="D64" s="15" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E64" s="15" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F64" s="15"/>
       <c r="G64" s="15"/>
@@ -3655,25 +3646,25 @@
       </c>
       <c r="O64" s="29"/>
       <c r="P64" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q64" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R64" s="29"/>
     </row>
     <row r="65" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C65" s="29" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E65" s="15" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F65" s="15" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G65" s="15"/>
       <c r="H65" s="30"/>
@@ -3687,20 +3678,20 @@
       </c>
       <c r="O65" s="29"/>
       <c r="P65" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q65" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R65" s="29"/>
     </row>
     <row r="66" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C66" s="29"/>
       <c r="D66" s="15" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="E66" s="15" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="F66" s="15"/>
       <c r="G66" s="15"/>
@@ -3714,19 +3705,19 @@
       <c r="O66" s="29"/>
       <c r="P66" s="38"/>
       <c r="Q66" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R66" s="29"/>
     </row>
     <row r="67" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C67" s="29" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D67" s="15" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E67" s="15" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="F67" s="15"/>
       <c r="G67" s="15"/>
@@ -3741,29 +3732,29 @@
       </c>
       <c r="O67" s="29"/>
       <c r="P67" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q67" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R67" s="29"/>
     </row>
     <row r="68" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C68" s="29" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D68" s="15" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E68" s="15" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="F68" s="15"/>
       <c r="G68" s="15"/>
       <c r="H68" s="30"/>
       <c r="I68" s="30"/>
       <c r="J68" s="15" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="K68" s="15"/>
       <c r="L68" s="15"/>
@@ -3773,10 +3764,10 @@
       </c>
       <c r="O68" s="29"/>
       <c r="P68" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q68" s="20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R68" s="29"/>
     </row>
@@ -3791,7 +3782,7 @@
       <c r="K69" s="1"/>
       <c r="L69" s="1"/>
       <c r="M69" s="32" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="70" spans="2:18" x14ac:dyDescent="0.25">
@@ -3807,7 +3798,7 @@
     </row>
     <row r="71" spans="2:18" ht="21" x14ac:dyDescent="0.35">
       <c r="D71" s="40" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E71" s="41"/>
       <c r="F71" s="41"/>
@@ -3820,7 +3811,7 @@
     </row>
     <row r="72" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C72" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D72" s="11" t="s">
         <v>1</v>
@@ -3829,14 +3820,14 @@
         <v>9</v>
       </c>
       <c r="F72" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G72" s="13"/>
       <c r="H72" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="I72" s="12" t="s">
         <v>77</v>
-      </c>
-      <c r="I72" s="12" t="s">
-        <v>78</v>
       </c>
       <c r="J72" s="11" t="s">
         <v>8</v>
@@ -3848,13 +3839,13 @@
         <v>20</v>
       </c>
       <c r="N72" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="O72" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="O72" s="12" t="s">
-        <v>80</v>
-      </c>
       <c r="P72" s="12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q72" s="1"/>
     </row>
@@ -3863,34 +3854,34 @@
         <v>55</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G73" s="1"/>
       <c r="H73" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I73" s="3"/>
       <c r="J73" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K73" s="22" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L73" s="1"/>
       <c r="N73" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P73" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q73" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="74" spans="2:18" x14ac:dyDescent="0.25">
@@ -3898,13 +3889,13 @@
         <v>55</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F74" s="33" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="G74" s="1"/>
       <c r="H74" s="3"/>
@@ -3913,13 +3904,13 @@
       <c r="K74" s="1"/>
       <c r="L74" s="1"/>
       <c r="N74" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P74" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q74" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="75" spans="2:18" x14ac:dyDescent="0.25">
@@ -3927,13 +3918,13 @@
         <v>55</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E75" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="F75" s="22" t="s">
         <v>208</v>
-      </c>
-      <c r="F75" s="22" t="s">
-        <v>211</v>
       </c>
       <c r="G75" s="1"/>
       <c r="H75" s="3"/>
@@ -3942,13 +3933,13 @@
       <c r="K75" s="1"/>
       <c r="L75" s="1"/>
       <c r="N75" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P75" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q75" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="76" spans="2:18" x14ac:dyDescent="0.25">
@@ -3956,13 +3947,13 @@
         <v>55</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F76" s="34" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="G76" s="1"/>
       <c r="H76" s="3"/>
@@ -3971,13 +3962,13 @@
       <c r="K76" s="1"/>
       <c r="L76" s="1"/>
       <c r="N76" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P76" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q76" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="77" spans="2:18" x14ac:dyDescent="0.25">
@@ -3985,13 +3976,13 @@
         <v>55</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F77" s="35" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="G77" s="1"/>
       <c r="H77" s="3"/>
@@ -4000,13 +3991,13 @@
       <c r="K77" s="1"/>
       <c r="L77" s="1"/>
       <c r="N77" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P77" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q77" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="78" spans="2:18" x14ac:dyDescent="0.25">
@@ -4014,13 +4005,13 @@
         <v>55</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F78" s="36" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="G78" s="1"/>
       <c r="H78" s="3"/>
@@ -4029,13 +4020,13 @@
       <c r="K78" s="1"/>
       <c r="L78" s="1"/>
       <c r="N78" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P78" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q78" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="79" spans="2:18" x14ac:dyDescent="0.25">
@@ -4046,13 +4037,13 @@
         <v>55</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="G79" s="1"/>
       <c r="H79" s="3"/>
@@ -4061,16 +4052,16 @@
       <c r="K79" s="1"/>
       <c r="L79" s="1"/>
       <c r="M79" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="N79" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P79" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q79" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="80" spans="2:18" x14ac:dyDescent="0.25">
@@ -4078,13 +4069,13 @@
         <v>55</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="G80" s="1"/>
       <c r="H80" s="3"/>
@@ -4093,13 +4084,13 @@
       <c r="K80" s="1"/>
       <c r="L80" s="1"/>
       <c r="N80" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P80" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q80" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="81" spans="3:17" x14ac:dyDescent="0.25">
@@ -4107,13 +4098,13 @@
         <v>55</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="G81" s="1"/>
       <c r="H81" s="37"/>
@@ -4122,13 +4113,13 @@
       <c r="K81" s="1"/>
       <c r="L81" s="1"/>
       <c r="N81" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P81" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q81" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="82" spans="3:17" x14ac:dyDescent="0.25">
@@ -4144,7 +4135,7 @@
     </row>
     <row r="83" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C83" s="32" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D83" s="1"/>
       <c r="E83" s="1"/>
@@ -4158,7 +4149,7 @@
     </row>
     <row r="84" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C84" s="32" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D84" s="1"/>
       <c r="E84" s="1"/>

</xml_diff>